<commit_message>
feat: push final docs
</commit_message>
<xml_diff>
--- a/docs/WBS_Helpdesk.xlsx
+++ b/docs/WBS_Helpdesk.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="181">
   <si>
     <t xml:space="preserve">WBS Aplikasi Helpdesk</t>
   </si>
   <si>
-    <t xml:space="preserve">Prioritas: Must = wajib untuk spesifikasi minimal; Should = melengkapi dan menambah nilai. Semua fitur pada daftar ini dikerjakan.</t>
+    <t xml:space="preserve">Prioritas: Must = wajib untuk spesifikasi minimal; Should = melengkapi dan menambah nilai. Status: 'Diimplementasikan' = sudah ada di repository; 'Rencana lanjutan' = direncanakan tetapi belum dikerjakan pada versi ini.</t>
   </si>
   <si>
     <t xml:space="preserve">Estimasi jam (teks biru) adalah perkiraan pribadi dan dapat diubah; subtotal dan total dihitung otomatis.</t>
@@ -504,6 +504,9 @@
   </si>
   <si>
     <t xml:space="preserve">Backend dapat diakses publik agar APK dan demo berfungsi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rencana lanjutan</t>
   </si>
   <si>
     <t xml:space="preserve">9</t>
@@ -2105,7 +2108,7 @@
         <v>14</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>15</v>
+        <v>161</v>
       </c>
       <c r="F58" s="9" t="n">
         <v>3</v>
@@ -2113,10 +2116,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C59" s="6"/>
       <c r="D59" s="6"/>
@@ -2128,13 +2131,13 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>14</v>
@@ -2148,13 +2151,13 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D61" s="7" t="s">
         <v>14</v>
@@ -2168,13 +2171,13 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>14</v>
@@ -2188,13 +2191,13 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D63" s="7" t="s">
         <v>22</v>
@@ -2209,7 +2212,7 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="10"/>
       <c r="B64" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C64" s="10"/>
       <c r="D64" s="10"/>
@@ -2247,7 +2250,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2255,10 +2258,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>14</v>
@@ -2464,10 +2467,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C12" s="13" t="n">
         <f aca="false">COUNTA(WBS!B60:B63)</f>
@@ -2489,7 +2492,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="17" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C13" s="16" t="n">
         <f aca="false">SUM(C4:C12)</f>

</xml_diff>